<commit_message>
continued work on README, added BOM and pictures.
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://draegerdeu-my.sharepoint.com/personal/jorn_koeppe_draeger_com/Documents/Desktop/THL/Scratchroboter/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://draegerdeu-my.sharepoint.com/personal/jorn_koeppe_draeger_com/Documents/Desktop/research/ASAPR/GitHub/ASAPR/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F5D3C189-AEB2-4655-80B1-79B7021FDCDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="91" documentId="8_{F5D3C189-AEB2-4655-80B1-79B7021FDCDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AA96BA6F-FAE4-4BF4-BBE6-A624BB1C8590}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-2805" windowWidth="29040" windowHeight="15720" xr2:uid="{0AA26A57-A96E-4AF8-AF19-1708DB280C07}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0AA26A57-A96E-4AF8-AF19-1708DB280C07}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="43">
   <si>
     <t>Component</t>
   </si>
@@ -68,18 +68,6 @@
     <t>Sourcing Link</t>
   </si>
   <si>
-    <t>Snapmaker A350®</t>
-  </si>
-  <si>
-    <t>SNAPMAKER HK LIMITED, Hong Kong</t>
-  </si>
-  <si>
-    <t>Industrial All-metal 3D Printer Online Sale – Snapmaker EU</t>
-  </si>
-  <si>
-    <t>3D-printer to perform the Scratch Assay and printing the used Parts(also other 3D-printers can be used, see GitHub)</t>
-  </si>
-  <si>
     <t>frame + slider</t>
   </si>
   <si>
@@ -89,49 +77,10 @@
     <t>GitHub(CAD files)</t>
   </si>
   <si>
-    <t>attachment block</t>
-  </si>
-  <si>
-    <t>block to attach the precision chuck directly to the printer(can only be used with SnapMaker A350)</t>
-  </si>
-  <si>
     <t xml:space="preserve">3D-printed part to fix the well on the print bed, ensuring the same postion time after time </t>
   </si>
   <si>
-    <t>M6 Adapter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adapter  for screwing pipette mount directly into M6 thread of any 3D printer </t>
-  </si>
-  <si>
-    <t>To be published</t>
-  </si>
-  <si>
-    <t>precision drill chuck</t>
-  </si>
-  <si>
-    <t xml:space="preserve">used to hold the the springloaded test probe </t>
-  </si>
-  <si>
-    <t>Donau Elektronik GmbH, Metten, germany</t>
-  </si>
-  <si>
-    <t>Bohrfutter 0,3-3,2 mm mit 2,35 mm Schaft Donau Elektronik MBS03 kaufen (conrad.de)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">clamps </t>
-  </si>
-  <si>
-    <t>clamps to fix the frame (Item 2) on the print bed</t>
-  </si>
-  <si>
     <t>FASBET</t>
-  </si>
-  <si>
-    <t>10 Stück 3D Drucker Heißbett Glasplattform Halter 3D Drucker Zubehör 3D Drucker Clip Klemme Zubehör 3D Drucker Heißbett Klemme für 3D-Drucker-Heißbett-Glasplatte Einstellbare Glas Halterung : Amazon.de: Gewerbe, Industrie &amp; Wissenschaft</t>
-  </si>
-  <si>
-    <t>pipette cutting device</t>
   </si>
   <si>
     <t>device for cutting pipettes to the same length repeatable</t>
@@ -165,13 +114,77 @@
       <t>€</t>
     </r>
   </si>
+  <si>
+    <t>3D-printed parts</t>
+  </si>
+  <si>
+    <t>M6 adapter</t>
+  </si>
+  <si>
+    <t>cutter</t>
+  </si>
+  <si>
+    <t>adapter for mounting the spring loaded (either with thread or without) test probe  to the printhead</t>
+  </si>
+  <si>
+    <t>parts to purchase</t>
+  </si>
+  <si>
+    <t>3D-printer</t>
+  </si>
+  <si>
+    <t>a FDM 3D-printer e.g. Snapmaker A350® or Prusa MK3S+®</t>
+  </si>
+  <si>
+    <t>depends</t>
+  </si>
+  <si>
+    <t>clamps</t>
+  </si>
+  <si>
+    <t>clamps to fix the frame (item 1) on the print bed</t>
+  </si>
+  <si>
+    <t>threaded insert</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M3 threaded insert (short) for the slider of the frame </t>
+  </si>
+  <si>
+    <t>CNC KITCHEN</t>
+  </si>
+  <si>
+    <t>M3 threaded insert</t>
+  </si>
+  <si>
+    <t>knurled knob</t>
+  </si>
+  <si>
+    <t>screw for the slider of the frame (goes into threaded insert)</t>
+  </si>
+  <si>
+    <t>Ganter</t>
+  </si>
+  <si>
+    <t>test probe</t>
+  </si>
+  <si>
+    <t>spring loaded test probe for holding the pipette (more information see README</t>
+  </si>
+  <si>
+    <t>INGUN Prüfmittelbau GmbH</t>
+  </si>
+  <si>
+    <t>Ingun</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="8" formatCode="#,##0.00\ &quot;€&quot;;[Red]\-#,##0.00\ &quot;€&quot;"/>
+    <numFmt numFmtId="165" formatCode="#,##0.000\ &quot;€&quot;;[Red]\-#,##0.000\ &quot;€&quot;"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -231,7 +244,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
@@ -240,6 +253,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -555,17 +569,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C073246-A4CD-4AD6-8AE5-D50E492FB90D}">
-  <dimension ref="A2:J13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A2:J19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="20.33203125" customWidth="1"/>
-    <col min="4" max="4" width="108.6640625" customWidth="1"/>
-    <col min="6" max="6" width="16.44140625" customWidth="1"/>
-    <col min="9" max="9" width="36.6640625" customWidth="1"/>
-    <col min="10" max="10" width="63.77734375" customWidth="1"/>
+    <col min="1" max="1" width="19.140625" customWidth="1"/>
+    <col min="3" max="3" width="23.85546875" customWidth="1"/>
+    <col min="4" max="4" width="108.7109375" customWidth="1"/>
+    <col min="6" max="6" width="16.42578125" customWidth="1"/>
+    <col min="9" max="9" width="36.7109375" customWidth="1"/>
+    <col min="10" max="10" width="63.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="4"/>
       <c r="B2" s="4" t="s">
         <v>1</v>
@@ -595,219 +610,281 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I5" t="s">
+        <v>11</v>
+      </c>
+      <c r="J5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B6">
         <v>2</v>
       </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="C6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="I6" t="s">
+        <v>11</v>
+      </c>
+      <c r="J6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B7">
+        <v>3</v>
+      </c>
+      <c r="C7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="I7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B10">
+        <v>4</v>
+      </c>
+      <c r="C10" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10" t="s">
+        <v>29</v>
+      </c>
+      <c r="H10" t="s">
+        <v>29</v>
+      </c>
+      <c r="I10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B11">
+        <v>5</v>
+      </c>
+      <c r="C11" t="s">
+        <v>32</v>
+      </c>
+      <c r="D11" t="s">
+        <v>33</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11">
+        <v>100</v>
+      </c>
+      <c r="G11" s="6">
+        <v>8.8999999999999996E-2</v>
+      </c>
+      <c r="H11" s="1">
+        <v>8.9</v>
+      </c>
+      <c r="I11" t="s">
+        <v>34</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B12">
+        <v>6</v>
+      </c>
+      <c r="C12" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" t="s">
+        <v>37</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12" s="1">
+        <v>0.95</v>
+      </c>
+      <c r="H12" s="1">
+        <v>0.95</v>
+      </c>
+      <c r="I12" t="s">
+        <v>38</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B13">
+        <v>7</v>
+      </c>
+      <c r="C13" t="s">
+        <v>30</v>
+      </c>
+      <c r="D13" t="s">
+        <v>31</v>
+      </c>
+      <c r="E13">
+        <v>4</v>
+      </c>
+      <c r="F13">
         <v>10</v>
       </c>
-      <c r="D4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-      <c r="G4" s="1">
-        <v>549</v>
-      </c>
-      <c r="H4" s="1">
-        <v>549</v>
-      </c>
-      <c r="I4" t="s">
-        <v>11</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B5">
-        <v>2</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="G13" s="1">
+        <v>0.8</v>
+      </c>
+      <c r="H13" s="1">
+        <v>7.99</v>
+      </c>
+      <c r="I13" t="s">
         <v>14</v>
       </c>
-      <c r="D5" t="s">
+      <c r="J13" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B14">
+        <v>8</v>
+      </c>
+      <c r="C14" t="s">
+        <v>39</v>
+      </c>
+      <c r="D14" t="s">
+        <v>40</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14" t="s">
+        <v>29</v>
+      </c>
+      <c r="H14" t="s">
+        <v>29</v>
+      </c>
+      <c r="I14" t="s">
+        <v>41</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15">
+        <v>9</v>
+      </c>
+      <c r="C15" t="s">
+        <v>17</v>
+      </c>
+      <c r="D15" t="s">
+        <v>18</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="H15">
+        <v>0</v>
+      </c>
+      <c r="J15" t="s">
         <v>19</v>
       </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="I5" t="s">
-        <v>15</v>
-      </c>
-      <c r="J5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B6">
-        <v>3</v>
-      </c>
-      <c r="C6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" t="s">
-        <v>28</v>
-      </c>
-      <c r="E6">
-        <v>4</v>
-      </c>
-      <c r="F6">
-        <v>10</v>
-      </c>
-      <c r="G6" s="1">
-        <v>0.8</v>
-      </c>
-      <c r="H6" s="1">
-        <v>7.99</v>
-      </c>
-      <c r="I6" t="s">
-        <v>29</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B7">
-        <v>4</v>
-      </c>
-      <c r="C7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" t="s">
-        <v>18</v>
-      </c>
-      <c r="E7">
-        <v>1</v>
-      </c>
-      <c r="F7">
-        <v>1</v>
-      </c>
-      <c r="I7" t="s">
-        <v>15</v>
-      </c>
-      <c r="J7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B8">
-        <v>5</v>
-      </c>
-      <c r="C8" t="s">
-        <v>23</v>
-      </c>
-      <c r="D8" t="s">
-        <v>24</v>
-      </c>
-      <c r="E8">
-        <v>1</v>
-      </c>
-      <c r="F8">
-        <v>1</v>
-      </c>
-      <c r="G8" s="1">
-        <v>9.9499999999999993</v>
-      </c>
-      <c r="H8" s="1">
-        <v>9.9499999999999993</v>
-      </c>
-      <c r="I8" t="s">
-        <v>25</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B9">
-        <v>6</v>
-      </c>
-      <c r="C9" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" t="s">
-        <v>21</v>
-      </c>
-      <c r="E9">
-        <v>1</v>
-      </c>
-      <c r="F9">
-        <v>1</v>
-      </c>
-      <c r="I9" t="s">
-        <v>15</v>
-      </c>
-      <c r="J9" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="B10">
-        <v>7</v>
-      </c>
-      <c r="C10" t="s">
-        <v>31</v>
-      </c>
-      <c r="D10" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A13" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B13">
-        <v>8</v>
-      </c>
-      <c r="C13" t="s">
-        <v>34</v>
-      </c>
-      <c r="D13" t="s">
-        <v>35</v>
-      </c>
-      <c r="E13">
-        <v>1</v>
-      </c>
-      <c r="F13">
-        <v>1</v>
-      </c>
-      <c r="G13">
-        <v>0</v>
-      </c>
-      <c r="H13">
-        <v>0</v>
-      </c>
-      <c r="J13" t="s">
-        <v>36</v>
-      </c>
+    </row>
+    <row r="19" spans="7:10" x14ac:dyDescent="0.25">
+      <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
+      <c r="J19" s="2"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="J4" r:id="rId1" display="https://eu.snapmaker.com/products/snapmaker-2-0-modular-3d-printer?variant=39620920279179&amp;gad_source=1&amp;gclid=Cj0KCQjwi5q3BhCiARIsAJCfuZnUwTBku8B-JENkTbG66b1JvGpSepBCLjGZJVko5btzOGIBoSg458saArfXEALw_wcB" xr:uid="{1BD2EC0B-12E8-4596-A6C3-D1125F4F4EC8}"/>
-    <hyperlink ref="J8" r:id="rId2" display="https://www.conrad.de/de/p/bohrfutter-0-3-3-2-mm-mit-2-35-mm-schaft-donau-elektronik-mbs03-2973401.html?refresh=true" xr:uid="{9B202FC5-2A1C-43E7-9306-AE32735E1BF2}"/>
-    <hyperlink ref="J6" r:id="rId3" display="https://www.amazon.de/Hei%C3%9Fbett-Glasplattform-3D-Drucker-Hei%C3%9Fbett-Glasplatte-Einstellbare-Halterung/dp/B0BVMGVBYK" xr:uid="{CBF3BF94-581F-4057-9674-28B357D48731}"/>
+    <hyperlink ref="J13" r:id="rId1" xr:uid="{CBF3BF94-581F-4057-9674-28B357D48731}"/>
+    <hyperlink ref="J11" r:id="rId2" xr:uid="{587DFCA2-082B-4571-8083-3E56C4F27A08}"/>
+    <hyperlink ref="J12" r:id="rId3" xr:uid="{691B7421-845D-47A4-B5CB-3ED997AEEE8C}"/>
+    <hyperlink ref="J14" r:id="rId4" xr:uid="{473898FF-02F8-4D4B-9D5F-748A5141ED14}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Arial"&amp;10&amp;KFF8F1F Internal&amp;1#_x000D_</oddHeader>
   </headerFooter>

</xml_diff>